<commit_message>
fix: normalize Excel - Riz blanc haricot -> Riz blanc, add Ursul Gurant + Kimie (88 commandes)
</commit_message>
<xml_diff>
--- a/linscrit.xlsx
+++ b/linscrit.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L87"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="16.81640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -648,7 +648,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -697,7 +697,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1040,7 +1040,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1515,7 +1515,7 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -3507,7 +3507,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
@@ -3561,7 +3561,7 @@
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3664,7 +3664,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -3772,7 +3772,7 @@
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Riz blanc haricot</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F81" t="inlineStr">
@@ -4722,7 +4722,7 @@
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Riz</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -4794,6 +4794,114 @@
         <v>86</v>
       </c>
       <c r="L87" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Ursul Gurant</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Individuel</t>
+        </is>
+      </c>
+      <c r="C88" t="n">
+        <v>1</v>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Bœuf</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Sur place</t>
+        </is>
+      </c>
+      <c r="H88" t="n">
+        <v>20</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>Non Payé</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>10</v>
+      </c>
+      <c r="K88" t="n">
+        <v>87</v>
+      </c>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>Non</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Kimie</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Individuel</t>
+        </is>
+      </c>
+      <c r="C89" t="n">
+        <v>1</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Travers de porc</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Sur place</t>
+        </is>
+      </c>
+      <c r="H89" t="n">
+        <v>10</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>Non Payé</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>10</v>
+      </c>
+      <c r="K89" t="n">
+        <v>88</v>
+      </c>
+      <c r="L89" t="inlineStr">
         <is>
           <t>Non</t>
         </is>

</xml_diff>

<commit_message>
fix: merge numbered entries into families (Tamara 6p, Sr Laurent 2p) + update Excel (82 rows)
</commit_message>
<xml_diff>
--- a/linscrit.xlsx
+++ b/linscrit.xlsx
@@ -552,7 +552,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L89"/>
+  <dimension ref="A1:L83"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="16.81640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Tamara 2</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1608,16 +1608,14 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C22" t="n">
+        <v>1</v>
+      </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>Bœuf</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -1632,10 +1630,10 @@
         </is>
       </c>
       <c r="J22" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1646,7 +1644,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Tamara 3</t>
+          <t>Famille Artiste</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1654,9 +1652,12 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C23" t="n">
+        <v>1</v>
+      </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1664,13 +1665,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>À emporter</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1678,10 +1684,10 @@
         </is>
       </c>
       <c r="J23" s="1" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1692,7 +1698,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Tamara 4</t>
+          <t>Famille Artiste</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1700,9 +1706,12 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C24" t="n">
+        <v>1</v>
+      </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1710,13 +1719,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>À emporter</t>
         </is>
       </c>
       <c r="H24" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
@@ -1724,10 +1738,10 @@
         </is>
       </c>
       <c r="J24" s="1" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1738,7 +1752,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Tamara 5</t>
+          <t>Famille Artiste</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1751,7 +1765,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1759,13 +1773,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>À emporter</t>
         </is>
       </c>
       <c r="H25" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
@@ -1773,10 +1792,10 @@
         </is>
       </c>
       <c r="J25" s="1" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1787,7 +1806,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Tamara 6</t>
+          <t>Sr Maricoise</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1800,7 +1819,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1808,13 +1827,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G26" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1822,10 +1846,10 @@
         </is>
       </c>
       <c r="J26" s="1" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1836,22 +1860,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Famille Julien</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>Famille</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
           <t>Bœuf</t>
         </is>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -1866,10 +1895,10 @@
         </is>
       </c>
       <c r="J27" s="1" t="n">
-        <v>20</v>
+        <v>119</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1880,7 +1909,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Famille Artiste</t>
+          <t>Famille Julien</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1888,9 +1917,6 @@
           <t>Individuel</t>
         </is>
       </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>Bœuf</t>
@@ -1901,18 +1927,13 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
@@ -1920,10 +1941,10 @@
         </is>
       </c>
       <c r="J28" s="1" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1934,7 +1955,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Famille Artiste</t>
+          <t>Famille Julien</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1942,9 +1963,6 @@
           <t>Individuel</t>
         </is>
       </c>
-      <c r="C29" t="n">
-        <v>1</v>
-      </c>
       <c r="D29" t="inlineStr">
         <is>
           <t>Bœuf</t>
@@ -1955,18 +1973,13 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
@@ -1974,10 +1987,10 @@
         </is>
       </c>
       <c r="J29" s="1" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -1988,7 +2001,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Famille Artiste</t>
+          <t>Famille Julien</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1996,12 +2009,9 @@
           <t>Individuel</t>
         </is>
       </c>
-      <c r="C30" t="n">
-        <v>1</v>
-      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Poulet fricassé</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -2009,18 +2019,13 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H30" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
@@ -2028,10 +2033,10 @@
         </is>
       </c>
       <c r="J30" s="1" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -2042,7 +2047,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Sr Maricoise</t>
+          <t>Famille Julien</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2050,12 +2055,9 @@
           <t>Individuel</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Poulet fricassé</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -2063,11 +2065,6 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G31" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -2082,10 +2079,10 @@
         </is>
       </c>
       <c r="J31" s="1" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2101,15 +2098,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Famille</t>
-        </is>
-      </c>
-      <c r="C32" t="n">
-        <v>7</v>
+          <t>Individuel</t>
+        </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2131,10 +2125,10 @@
         </is>
       </c>
       <c r="J32" s="1" t="n">
-        <v>119</v>
+        <v>0</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2155,7 +2149,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -2180,7 +2174,7 @@
         <v>0</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2191,7 +2185,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Fr Laurent</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2199,14 +2193,17 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C34" t="n">
+        <v>1</v>
+      </c>
       <c r="D34" t="inlineStr">
         <is>
           <t>Bœuf</t>
         </is>
       </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2223,10 +2220,10 @@
         </is>
       </c>
       <c r="J34" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -2237,22 +2234,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Sr Laurent</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Individuel</t>
-        </is>
+          <t>Famille</t>
+        </is>
+      </c>
+      <c r="C35" t="n">
+        <v>2</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
+          <t>Bœuf</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2269,10 +2269,10 @@
         </is>
       </c>
       <c r="J35" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2283,7 +2283,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Famille Léa</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2291,9 +2291,12 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C36" t="n">
+        <v>1</v>
+      </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -2315,10 +2318,10 @@
         </is>
       </c>
       <c r="J36" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2329,7 +2332,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Famille Léa</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2337,9 +2340,12 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C37" t="n">
+        <v>1</v>
+      </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -2361,10 +2367,10 @@
         </is>
       </c>
       <c r="J37" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>36</v>
+        <v>41</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2375,7 +2381,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Famille Léa</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -2383,14 +2389,17 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C38" t="n">
+        <v>1</v>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Gratin de banane</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2407,10 +2416,10 @@
         </is>
       </c>
       <c r="J38" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2421,7 +2430,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Fr Laurent</t>
+          <t>Sr Petit Frère</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -2434,21 +2443,21 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Travers de porc</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>À emporter</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2456,10 +2465,10 @@
         </is>
       </c>
       <c r="J39" s="1" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>38</v>
+        <v>43</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2470,7 +2479,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sr Laurent</t>
+          <t>Moricia</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -2486,18 +2495,18 @@
           <t>Bœuf</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>À emporter</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2505,10 +2514,10 @@
         </is>
       </c>
       <c r="J40" s="1" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2519,7 +2528,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Famille Léa</t>
+          <t>Odette</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2542,11 +2551,11 @@
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>À emporter</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2554,10 +2563,10 @@
         </is>
       </c>
       <c r="J41" s="1" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2568,7 +2577,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Famille Léa</t>
+          <t>Sr Françoise</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2581,7 +2590,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Poulet fricassé</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -2589,6 +2598,11 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -2606,7 +2620,7 @@
         <v>20</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2617,7 +2631,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Famille Léa</t>
+          <t>Sr Françoise</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -2630,12 +2644,17 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Poulet fricassé</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz collé</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2655,7 +2674,7 @@
         <v>20</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2666,7 +2685,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sr Petit Frère</t>
+          <t>Sr Toussaint</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2679,7 +2698,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2689,11 +2708,11 @@
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2701,10 +2720,10 @@
         </is>
       </c>
       <c r="J44" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2715,7 +2734,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Moricia</t>
+          <t>Roseline</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2728,7 +2747,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -2736,13 +2755,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H45" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
@@ -2750,10 +2774,10 @@
         </is>
       </c>
       <c r="J45" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2764,7 +2788,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Odette</t>
+          <t>Roseline</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2782,16 +2806,21 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Gratin de banane</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H46" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2799,10 +2828,10 @@
         </is>
       </c>
       <c r="J46" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -2813,7 +2842,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Sr Françoise</t>
+          <t>Marie Carnouche</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2826,17 +2855,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Travers de porc</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F47" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Gratin de banane</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2856,7 +2880,7 @@
         <v>20</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -2867,7 +2891,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sr Françoise</t>
+          <t>Raymonde</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -2885,12 +2909,7 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F48" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Gratin de banane</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2910,7 +2929,7 @@
         <v>20</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -2921,7 +2940,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Sr Toussaint</t>
+          <t>Famille Georges</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -2932,16 +2951,6 @@
       <c r="C49" t="n">
         <v>1</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E49" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
       <c r="G49" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -2959,7 +2968,7 @@
         <v>20</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
@@ -2970,7 +2979,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Roseline</t>
+          <t>Famille Georges</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2981,21 +2990,6 @@
       <c r="C50" t="n">
         <v>1</v>
       </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E50" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F50" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G50" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -3013,7 +3007,7 @@
         <v>20</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -3024,7 +3018,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Roseline</t>
+          <t>Famille Georges</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -3035,21 +3029,6 @@
       <c r="C51" t="n">
         <v>1</v>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Gratin de banane</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G51" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -3067,7 +3046,7 @@
         <v>20</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
@@ -3078,7 +3057,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Marie Carnouche</t>
+          <t>Serina</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3091,12 +3070,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Poulet fricassé</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -3116,7 +3095,7 @@
         <v>20</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
@@ -3127,7 +3106,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Raymonde</t>
+          <t>Beaudelaire</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -3140,12 +3119,12 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -3165,7 +3144,7 @@
         <v>20</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
@@ -3176,7 +3155,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Famille Georges</t>
+          <t>Marcelin Chaarlie</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -3187,6 +3166,16 @@
       <c r="C54" t="n">
         <v>1</v>
       </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Crevette sauce poivrée</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
       <c r="G54" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -3204,7 +3193,7 @@
         <v>20</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -3215,7 +3204,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Famille Georges</t>
+          <t>Claunette</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3226,13 +3215,23 @@
       <c r="C55" t="n">
         <v>1</v>
       </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Bœuf</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
       <c r="G55" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H55" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I55" t="inlineStr">
         <is>
@@ -3240,10 +3239,10 @@
         </is>
       </c>
       <c r="J55" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
@@ -3254,7 +3253,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Famille Georges</t>
+          <t>Pierre Laurole</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -3265,6 +3264,21 @@
       <c r="C56" t="n">
         <v>1</v>
       </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Bœuf</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G56" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -3282,7 +3296,7 @@
         <v>20</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
@@ -3293,7 +3307,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Serina</t>
+          <t>Margarette</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -3306,7 +3320,7 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
@@ -3331,7 +3345,7 @@
         <v>20</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
@@ -3342,7 +3356,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Beaudelaire</t>
+          <t>Mathias</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3355,7 +3369,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -3363,6 +3377,11 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G58" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -3380,7 +3399,7 @@
         <v>20</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -3391,7 +3410,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Marcelin Chaarlie</t>
+          <t>Gladys</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -3404,12 +3423,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Travers de porc</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -3418,7 +3442,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I59" t="inlineStr">
         <is>
@@ -3426,10 +3450,10 @@
         </is>
       </c>
       <c r="J59" s="1" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
@@ -3440,7 +3464,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Claunette</t>
+          <t>Lacia</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -3461,13 +3485,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G60" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H60" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="I60" t="inlineStr">
         <is>
@@ -3475,10 +3504,10 @@
         </is>
       </c>
       <c r="J60" s="1" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="L60" t="inlineStr">
         <is>
@@ -3489,7 +3518,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Pierre Laurole</t>
+          <t>Clozel</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -3502,7 +3531,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
@@ -3521,7 +3550,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I61" t="inlineStr">
         <is>
@@ -3529,10 +3558,10 @@
         </is>
       </c>
       <c r="J61" s="1" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="L61" t="inlineStr">
         <is>
@@ -3543,7 +3572,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Margarette</t>
+          <t>Edwin</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -3556,12 +3585,12 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Travers de porc</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -3581,7 +3610,7 @@
         <v>20</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -3592,7 +3621,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Mathias</t>
+          <t>Gina</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -3605,17 +3634,12 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Gratin de banane</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -3624,7 +3648,7 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I63" t="inlineStr">
         <is>
@@ -3632,10 +3656,10 @@
         </is>
       </c>
       <c r="J63" s="1" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
@@ -3646,7 +3670,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Gladys</t>
+          <t>Ocema</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -3659,17 +3683,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Calalou</t>
+          <t>Haricot vert</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -3689,7 +3713,7 @@
         <v>0</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -3700,7 +3724,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Lacia</t>
+          <t>Eloise Bruno</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -3710,21 +3734,6 @@
       </c>
       <c r="C65" t="n">
         <v>1</v>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E65" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F65" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
       </c>
       <c r="G65" t="inlineStr">
         <is>
@@ -3743,7 +3752,7 @@
         <v>0</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
@@ -3754,39 +3763,24 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Clozel</t>
+          <t>Lézimène</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>Famille</t>
         </is>
       </c>
       <c r="C66" t="n">
         <v>1</v>
       </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F66" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G66" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H66" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I66" t="inlineStr">
         <is>
@@ -3794,10 +3788,10 @@
         </is>
       </c>
       <c r="J66" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
@@ -3808,7 +3802,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Edwin</t>
+          <t>Chloé</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -3819,16 +3813,6 @@
       <c r="C67" t="n">
         <v>1</v>
       </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
       <c r="G67" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -3846,7 +3830,7 @@
         <v>20</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
@@ -3857,7 +3841,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Gina</t>
+          <t>Mr Bruno</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -3868,14 +3852,9 @@
       <c r="C68" t="n">
         <v>1</v>
       </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -3884,7 +3863,7 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I68" t="inlineStr">
         <is>
@@ -3892,10 +3871,10 @@
         </is>
       </c>
       <c r="J68" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -3906,7 +3885,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Ocema</t>
+          <t>Madame Bruno</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -3917,28 +3896,13 @@
       <c r="C69" t="n">
         <v>1</v>
       </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F69" t="inlineStr">
-        <is>
-          <t>Haricot vert</t>
-        </is>
-      </c>
       <c r="G69" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H69" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I69" t="inlineStr">
         <is>
@@ -3946,10 +3910,10 @@
         </is>
       </c>
       <c r="J69" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
@@ -3960,7 +3924,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Eloise Bruno</t>
+          <t>Madcène</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -3977,7 +3941,7 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I70" t="inlineStr">
         <is>
@@ -3985,10 +3949,10 @@
         </is>
       </c>
       <c r="J70" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
@@ -3999,12 +3963,12 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>Lézimène</t>
+          <t>Madina</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>Individuel</t>
         </is>
       </c>
       <c r="C71" t="n">
@@ -4027,7 +3991,7 @@
         <v>20</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
@@ -4038,7 +4002,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>Chloé</t>
+          <t>Ermie</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4049,13 +4013,28 @@
       <c r="C72" t="n">
         <v>1</v>
       </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Poulet fricassé</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G72" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H72" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I72" t="inlineStr">
         <is>
@@ -4063,10 +4042,10 @@
         </is>
       </c>
       <c r="J72" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
@@ -4077,7 +4056,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Mr Bruno</t>
+          <t>Numa Marie</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4088,9 +4067,19 @@
       <c r="C73" t="n">
         <v>1</v>
       </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Bœuf</t>
+        </is>
+      </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
+          <t>Riz collé</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -4110,7 +4099,7 @@
         <v>20</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
@@ -4121,7 +4110,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Madame Bruno</t>
+          <t>Johnson</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4132,6 +4121,21 @@
       <c r="C74" t="n">
         <v>1</v>
       </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Poulet fricassé</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G74" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -4149,7 +4153,7 @@
         <v>20</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="L74" t="inlineStr">
         <is>
@@ -4160,7 +4164,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Madcène</t>
+          <t>Medson</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4171,13 +4175,28 @@
       <c r="C75" t="n">
         <v>1</v>
       </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Travers de porc</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Haricot vert</t>
+        </is>
+      </c>
       <c r="G75" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H75" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I75" t="inlineStr">
         <is>
@@ -4185,10 +4204,10 @@
         </is>
       </c>
       <c r="J75" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="L75" t="inlineStr">
         <is>
@@ -4199,7 +4218,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Madina</t>
+          <t>Sheskah</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4210,6 +4229,21 @@
       <c r="C76" t="n">
         <v>1</v>
       </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>Crevette sauce poivrée</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G76" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -4227,7 +4261,7 @@
         <v>20</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
@@ -4238,7 +4272,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Ermie</t>
+          <t>Hélène Jean</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4251,17 +4285,17 @@
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t>Calalou</t>
+          <t>Haricot vert</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -4281,7 +4315,7 @@
         <v>10</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
@@ -4292,7 +4326,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Numa Marie</t>
+          <t>Maman Lésimène</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4305,17 +4339,7 @@
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E78" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F78" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Travers de porc</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -4335,7 +4359,7 @@
         <v>20</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
@@ -4346,7 +4370,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Johnson</t>
+          <t>Rita Pierre</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4359,12 +4383,7 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E79" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -4389,7 +4408,7 @@
         <v>20</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
@@ -4400,30 +4419,25 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Medson</t>
+          <t>Maturin</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>Famille</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F80" t="inlineStr">
-        <is>
-          <t>Haricot vert</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -4432,7 +4446,7 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="I80" t="inlineStr">
         <is>
@@ -4440,10 +4454,10 @@
         </is>
       </c>
       <c r="J80" s="1" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
@@ -4454,7 +4468,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Sheskah</t>
+          <t>Jean-Baptiste</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4467,17 +4481,12 @@
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Travers de porc</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F81" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -4486,7 +4495,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I81" t="inlineStr">
         <is>
@@ -4494,10 +4503,10 @@
         </is>
       </c>
       <c r="J81" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
@@ -4508,7 +4517,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Hélène Jean</t>
+          <t>Ursul Gurant</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4521,17 +4530,17 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>Haricot vert</t>
+          <t>Calalou</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -4540,18 +4549,18 @@
         </is>
       </c>
       <c r="H82" t="n">
+        <v>20</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>Non Payé</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
         <v>10</v>
       </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J82" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K82" s="2" t="n">
-        <v>81</v>
+      <c r="K82" t="n">
+        <v>87</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
@@ -4562,7 +4571,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Maman Lésimène</t>
+          <t>Kimie</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4578,330 +4587,36 @@
           <t>Travers de porc</t>
         </is>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Calalou</t>
+        </is>
+      </c>
       <c r="G83" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H83" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I83" t="inlineStr">
         <is>
           <t>Non Payé</t>
         </is>
       </c>
-      <c r="J83" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K83" s="2" t="n">
-        <v>82</v>
+      <c r="J83" t="n">
+        <v>10</v>
+      </c>
+      <c r="K83" t="n">
+        <v>88</v>
       </c>
       <c r="L83" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>Sr Laurent 2</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C84" t="n">
-        <v>1</v>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="F84" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H84" t="n">
-        <v>20</v>
-      </c>
-      <c r="I84" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J84" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K84" s="2" t="n">
-        <v>83</v>
-      </c>
-      <c r="L84" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>Rita Pierre</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C85" t="n">
-        <v>1</v>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="F85" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H85" t="n">
-        <v>20</v>
-      </c>
-      <c r="I85" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J85" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K85" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="L85" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>Maturin</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>Famille</t>
-        </is>
-      </c>
-      <c r="C86" t="n">
-        <v>2</v>
-      </c>
-      <c r="D86" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E86" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H86" t="n">
-        <v>20</v>
-      </c>
-      <c r="I86" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J86" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="K86" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="L86" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>Jean-Baptiste</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C87" t="n">
-        <v>1</v>
-      </c>
-      <c r="D87" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E87" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H87" t="n">
-        <v>10</v>
-      </c>
-      <c r="I87" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J87" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K87" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="L87" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>Ursul Gurant</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C88" t="n">
-        <v>1</v>
-      </c>
-      <c r="D88" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F88" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H88" t="n">
-        <v>20</v>
-      </c>
-      <c r="I88" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J88" t="n">
-        <v>10</v>
-      </c>
-      <c r="K88" t="n">
-        <v>87</v>
-      </c>
-      <c r="L88" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>Kimie</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C89" t="n">
-        <v>1</v>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E89" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F89" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H89" t="n">
-        <v>10</v>
-      </c>
-      <c r="I89" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J89" t="n">
-        <v>10</v>
-      </c>
-      <c r="K89" t="n">
-        <v>88</v>
-      </c>
-      <c r="L89" t="inlineStr">
         <is>
           <t>Non</t>
         </is>

</xml_diff>

<commit_message>
Excel: merge familles (Laurole+Ursule, Pierre Louis, Bourdeau, Gabriel, Doisy, Gaspard, Tamara, Artiste, Julien, Laurent, Lea, Francoise, Roseline, Georges, Luxama, Bruno, Lezimene), normalise Riz blanc, supprime enfants absorbes, Jacotin=4p, Kimie supprimee
</commit_message>
<xml_diff>
--- a/linscrit.xlsx
+++ b/linscrit.xlsx
@@ -19,7 +19,7 @@
     <definedName name="type">[1]paramètres!$E$3:$E$4</definedName>
     <definedName name="viande">[1]paramètres!$A$3:$A$6</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -66,7 +66,12 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="2">
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+    </dxf>
     <dxf>
       <font>
         <color rgb="FFFF0000"/>
@@ -552,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L83"/>
+  <dimension ref="A1:L48"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5"/>
   <cols>
     <col width="16.81640625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -635,7 +640,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -684,7 +689,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -692,7 +697,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -702,7 +707,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>A emporter</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -728,16 +733,16 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Gaspard Daphose</t>
+          <t>Famille Gaspard</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -777,7 +782,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Gaspard Byalone</t>
+          <t>Evelyne</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -790,21 +795,21 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>A emporter</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -812,10 +817,10 @@
         </is>
       </c>
       <c r="J5" s="1" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="L5" t="inlineStr">
         <is>
@@ -826,7 +831,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Evelyne</t>
+          <t>Rosina</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -839,21 +844,21 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -861,10 +866,10 @@
         </is>
       </c>
       <c r="J6" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
@@ -875,7 +880,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Rosina</t>
+          <t>Dorval Mamouna</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -888,12 +893,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Travers de Porc</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -913,7 +918,7 @@
         <v>20</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
@@ -924,7 +929,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Dorval Mamouna</t>
+          <t>Bossé Tiroulio</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -937,7 +942,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -962,7 +967,7 @@
         <v>20</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -973,7 +978,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Bossé Tiroulio</t>
+          <t>Merena</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -986,12 +991,17 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -1011,7 +1021,7 @@
         <v>20</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L9" t="inlineStr">
         <is>
@@ -1022,30 +1032,25 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Merena</t>
+          <t>Famille Jacotin</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -1062,10 +1067,10 @@
         </is>
       </c>
       <c r="J10" s="1" t="n">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
@@ -1076,20 +1081,20 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Famille Jacotin</t>
+          <t>Jonas</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>Individuel</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1111,10 +1116,10 @@
         </is>
       </c>
       <c r="J11" s="1" t="n">
-        <v>60</v>
+        <v>20</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
@@ -1125,7 +1130,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Jonas</t>
+          <t>Judith</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -1138,12 +1143,12 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Gratin de Banane</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1163,7 +1168,7 @@
         <v>20</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
@@ -1174,25 +1179,20 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Judith</t>
+          <t>Famille Gabriel</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>Gratin de banane</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1212,7 +1212,7 @@
         <v>20</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
@@ -1223,20 +1223,20 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Fr Gabriel</t>
+          <t>Famille Doisy</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1256,7 +1256,7 @@
         <v>20</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
@@ -1267,7 +1267,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Sr Gabriel</t>
+          <t>Sr Mervil</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1300,7 +1300,7 @@
         <v>20</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
@@ -1311,20 +1311,25 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Fr Doisy</t>
+          <t>Famille Pierre Louis</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>Bœuf</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1344,7 +1349,7 @@
         <v>20</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
@@ -1355,25 +1360,25 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Sr Doisy</t>
+          <t>Famille Tamara</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
           <t>Bœuf</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1390,10 +1395,10 @@
         </is>
       </c>
       <c r="J17" s="1" t="n">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
@@ -1404,7 +1409,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Sr Mervil</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1417,7 +1422,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Bœuf</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1437,7 +1442,7 @@
         <v>20</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>17</v>
+        <v>26</v>
       </c>
       <c r="L18" t="inlineStr">
         <is>
@@ -1448,16 +1453,16 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Marenn Pierre Louis</t>
+          <t>Famille Artiste</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -1469,13 +1474,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>calalou</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>A emporter</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1483,10 +1493,10 @@
         </is>
       </c>
       <c r="J19" s="1" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
@@ -1497,7 +1507,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Pierre Louis</t>
+          <t>Sr maricoise</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1515,12 +1525,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>Riz blanc</t>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Calalou</t>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1540,7 +1550,7 @@
         <v>20</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
@@ -1551,16 +1561,16 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Famille Tamara</t>
+          <t>Famille Julien</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -1586,10 +1596,10 @@
         </is>
       </c>
       <c r="J21" s="1" t="n">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>20</v>
+        <v>31</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
@@ -1600,22 +1610,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mode</t>
+          <t>Famille Laurent</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
           <t>Bœuf</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>calalou</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -1633,7 +1648,7 @@
         <v>20</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
@@ -1644,16 +1659,16 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Famille Artiste</t>
+          <t>Famille Léa</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
@@ -1665,18 +1680,13 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -1684,10 +1694,10 @@
         </is>
       </c>
       <c r="J23" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="L23" t="inlineStr">
         <is>
@@ -1698,7 +1708,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Famille Artiste</t>
+          <t>sr Petit frère</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1711,7 +1721,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Travers de Porc</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -1719,14 +1729,9 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>A emporter</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -1741,7 +1746,7 @@
         <v>15</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>28</v>
+        <v>43</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
@@ -1752,7 +1757,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Famille Artiste</t>
+          <t>Moricia</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1773,14 +1778,9 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>A emporter</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -1795,7 +1795,7 @@
         <v>15</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>29</v>
+        <v>44</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
@@ -1806,7 +1806,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Sr Maricoise</t>
+          <t>Odette</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1827,18 +1827,13 @@
           <t>Riz collé</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Sur place</t>
+          <t>A emporter</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -1846,10 +1841,10 @@
         </is>
       </c>
       <c r="J26" s="1" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
@@ -1860,20 +1855,20 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Famille Françoise</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1881,6 +1876,11 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>calalou</t>
+        </is>
+      </c>
       <c r="G27" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -1895,10 +1895,10 @@
         </is>
       </c>
       <c r="J27" s="1" t="n">
-        <v>119</v>
+        <v>20</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
@@ -1909,7 +1909,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>sr Toussaint</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1917,6 +1917,9 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C28" t="n">
+        <v>1</v>
+      </c>
       <c r="D28" t="inlineStr">
         <is>
           <t>Bœuf</t>
@@ -1941,10 +1944,10 @@
         </is>
       </c>
       <c r="J28" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>32</v>
+        <v>48</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
@@ -1955,17 +1958,20 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Famille Roseline</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Individuel</t>
-        </is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1973,6 +1979,11 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>calalou</t>
+        </is>
+      </c>
       <c r="G29" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -1987,10 +1998,10 @@
         </is>
       </c>
       <c r="J29" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>33</v>
+        <v>49</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
@@ -2001,7 +2012,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Marie Carnouche</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -2009,14 +2020,17 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C30" t="n">
+        <v>1</v>
+      </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Travers de Porc</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Gratin de Banane</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2033,10 +2047,10 @@
         </is>
       </c>
       <c r="J30" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
@@ -2047,7 +2061,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Raymonde</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -2055,14 +2069,17 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Gratin de Banane</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2079,10 +2096,10 @@
         </is>
       </c>
       <c r="J31" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>35</v>
+        <v>52</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
@@ -2093,23 +2110,16 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Famille Georges</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="D32" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
+          <t>famille</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -2125,10 +2135,10 @@
         </is>
       </c>
       <c r="J32" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="L32" t="inlineStr">
         <is>
@@ -2139,7 +2149,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Famille Julien</t>
+          <t>Serina</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2147,14 +2157,17 @@
           <t>Individuel</t>
         </is>
       </c>
+      <c r="C33" t="n">
+        <v>1</v>
+      </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Crevette sauce poivrée</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2171,10 +2184,10 @@
         </is>
       </c>
       <c r="J33" s="1" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="L33" t="inlineStr">
         <is>
@@ -2185,7 +2198,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Fr Laurent</t>
+          <t>Beaudelaire</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -2198,12 +2211,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Crevette sauce poivrée</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2223,7 +2236,7 @@
         <v>20</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
@@ -2234,25 +2247,25 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Sr Laurent</t>
+          <t>Marcelin Chaarlie</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Famille</t>
+          <t>Individuel</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>Calalou</t>
+          <t>Crevette sauce poivrée</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Riz collé</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2272,7 +2285,7 @@
         <v>20</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
@@ -2283,7 +2296,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Famille Léa</t>
+          <t>Claunette</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -2310,7 +2323,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
@@ -2318,10 +2331,10 @@
         </is>
       </c>
       <c r="J36" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="L36" t="inlineStr">
         <is>
@@ -2332,16 +2345,16 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Famille Léa</t>
+          <t>Famille Laurole</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
@@ -2350,7 +2363,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2370,7 +2388,7 @@
         <v>20</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="L37" t="inlineStr">
         <is>
@@ -2381,25 +2399,30 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Famille Léa</t>
+          <t>Famille Luxama</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Travers de Porc</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz blanc</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -2408,7 +2431,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
@@ -2416,10 +2439,10 @@
         </is>
       </c>
       <c r="J38" s="1" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>42</v>
+        <v>63</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
@@ -2430,34 +2453,34 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Sr Petit Frère</t>
+          <t>Famille Bruno</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Gratin de Banane</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H39" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
@@ -2465,10 +2488,10 @@
         </is>
       </c>
       <c r="J39" s="1" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
@@ -2479,34 +2502,24 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Moricia</t>
+          <t>Famille Lézimène</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>Famille</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>1</v>
-      </c>
-      <c r="D40" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
+        <v>3</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H40" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
@@ -2514,10 +2527,10 @@
         </is>
       </c>
       <c r="J40" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>44</v>
+        <v>70</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
@@ -2528,7 +2541,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Odette</t>
+          <t>Madcène</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2539,23 +2552,13 @@
       <c r="C41" t="n">
         <v>1</v>
       </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>À emporter</t>
+          <t>Sur place</t>
         </is>
       </c>
       <c r="H41" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
@@ -2563,10 +2566,10 @@
         </is>
       </c>
       <c r="J41" s="1" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>45</v>
+        <v>74</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
@@ -2577,7 +2580,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Sr Françoise</t>
+          <t>Madina</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -2588,21 +2591,6 @@
       <c r="C42" t="n">
         <v>1</v>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
       <c r="G42" t="inlineStr">
         <is>
           <t>Sur place</t>
@@ -2620,7 +2608,7 @@
         <v>20</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>46</v>
+        <v>75</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
@@ -2631,20 +2619,20 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Sr Françoise</t>
+          <t>Famille Bourdeau</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>poulet fricassé</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -2654,7 +2642,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Calalou</t>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -2663,7 +2651,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
@@ -2671,10 +2659,10 @@
         </is>
       </c>
       <c r="J43" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>47</v>
+        <v>76</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
@@ -2685,7 +2673,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Sr Toussaint</t>
+          <t>Medson</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -2698,7 +2686,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Travers de Porc</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -2706,13 +2694,18 @@
           <t>Riz collé</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Haricot vert</t>
+        </is>
+      </c>
       <c r="G44" t="inlineStr">
         <is>
           <t>Sur place</t>
         </is>
       </c>
       <c r="H44" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
@@ -2720,10 +2713,10 @@
         </is>
       </c>
       <c r="J44" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>48</v>
+        <v>79</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
@@ -2734,7 +2727,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Roseline</t>
+          <t>Sheskah</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -2752,12 +2745,12 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>Riz collé</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Calalou</t>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -2777,7 +2770,7 @@
         <v>20</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
@@ -2788,7 +2781,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Roseline</t>
+          <t>Hélène jean</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -2801,17 +2794,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Bœuf</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Calalou</t>
+          <t>Haricot vert</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -2820,7 +2813,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
@@ -2828,10 +2821,10 @@
         </is>
       </c>
       <c r="J46" s="1" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>50</v>
+        <v>81</v>
       </c>
       <c r="L46" t="inlineStr">
         <is>
@@ -2842,7 +2835,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Marie Carnouche</t>
+          <t>Rita Pierre</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -2855,12 +2848,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>Gratin de banane</t>
+          <t>Bœuf</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>calalou</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -2880,7 +2873,7 @@
         <v>20</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>51</v>
+        <v>84</v>
       </c>
       <c r="L47" t="inlineStr">
         <is>
@@ -2891,25 +2884,25 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Raymonde</t>
+          <t>maturin</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Individuel</t>
+          <t>famille</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Poulet fricassé</t>
+          <t>Crevette sauce poivrée</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Gratin de banane</t>
+          <t>Riz blanc</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -2926,10 +2919,10 @@
         </is>
       </c>
       <c r="J48" s="1" t="n">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>52</v>
+        <v>85</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -2937,1693 +2930,8 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
-        <is>
-          <t>Famille Georges</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H49" t="n">
-        <v>20</v>
-      </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J49" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K49" s="2" t="n">
-        <v>53</v>
-      </c>
-      <c r="L49" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>Famille Georges</t>
-        </is>
-      </c>
-      <c r="B50" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C50" t="n">
-        <v>1</v>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H50" t="n">
-        <v>20</v>
-      </c>
-      <c r="I50" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J50" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K50" s="2" t="n">
-        <v>54</v>
-      </c>
-      <c r="L50" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>Famille Georges</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>20</v>
-      </c>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J51" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K51" s="2" t="n">
-        <v>55</v>
-      </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="52">
-      <c r="A52" t="inlineStr">
-        <is>
-          <t>Serina</t>
-        </is>
-      </c>
-      <c r="B52" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C52" t="n">
-        <v>1</v>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E52" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H52" t="n">
-        <v>20</v>
-      </c>
-      <c r="I52" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J52" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K52" s="2" t="n">
-        <v>56</v>
-      </c>
-      <c r="L52" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>Beaudelaire</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C53" t="n">
-        <v>1</v>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>20</v>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J53" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K53" s="2" t="n">
-        <v>57</v>
-      </c>
-      <c r="L53" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>Marcelin Chaarlie</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>1</v>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H54" t="n">
-        <v>20</v>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J54" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K54" s="2" t="n">
-        <v>58</v>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>Claunette</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C55" t="n">
-        <v>1</v>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H55" t="n">
-        <v>10</v>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J55" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K55" s="2" t="n">
-        <v>59</v>
-      </c>
-      <c r="L55" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>Pierre Laurole</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C56" t="n">
-        <v>1</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H56" t="n">
-        <v>20</v>
-      </c>
-      <c r="I56" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J56" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K56" s="2" t="n">
-        <v>60</v>
-      </c>
-      <c r="L56" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Margarette</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C57" t="n">
-        <v>1</v>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E57" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H57" t="n">
-        <v>20</v>
-      </c>
-      <c r="I57" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J57" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K57" s="2" t="n">
-        <v>61</v>
-      </c>
-      <c r="L57" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>Mathias</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C58" t="n">
-        <v>1</v>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E58" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F58" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H58" t="n">
-        <v>20</v>
-      </c>
-      <c r="I58" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J58" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K58" s="2" t="n">
-        <v>62</v>
-      </c>
-      <c r="L58" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Gladys</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F59" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H59" t="n">
-        <v>0</v>
-      </c>
-      <c r="I59" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J59" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K59" s="2" t="n">
-        <v>63</v>
-      </c>
-      <c r="L59" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>Lacia</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C60" t="n">
-        <v>1</v>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F60" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H60" t="n">
-        <v>0</v>
-      </c>
-      <c r="I60" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J60" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K60" s="2" t="n">
-        <v>64</v>
-      </c>
-      <c r="L60" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>Clozel</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C61" t="n">
-        <v>1</v>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E61" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H61" t="n">
-        <v>0</v>
-      </c>
-      <c r="I61" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J61" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K61" s="2" t="n">
-        <v>65</v>
-      </c>
-      <c r="L61" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>Edwin</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C62" t="n">
-        <v>1</v>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H62" t="n">
-        <v>20</v>
-      </c>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J62" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K62" s="2" t="n">
-        <v>66</v>
-      </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>Gina</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C63" t="n">
-        <v>1</v>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Gratin de banane</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H63" t="n">
-        <v>0</v>
-      </c>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J63" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K63" s="2" t="n">
-        <v>67</v>
-      </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>Ocema</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C64" t="n">
-        <v>1</v>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F64" t="inlineStr">
-        <is>
-          <t>Haricot vert</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H64" t="n">
-        <v>0</v>
-      </c>
-      <c r="I64" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J64" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K64" s="2" t="n">
-        <v>68</v>
-      </c>
-      <c r="L64" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>Eloise Bruno</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C65" t="n">
-        <v>1</v>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H65" t="n">
-        <v>0</v>
-      </c>
-      <c r="I65" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J65" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="K65" s="2" t="n">
-        <v>69</v>
-      </c>
-      <c r="L65" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>Lézimène</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>Famille</t>
-        </is>
-      </c>
-      <c r="C66" t="n">
-        <v>1</v>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H66" t="n">
-        <v>20</v>
-      </c>
-      <c r="I66" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J66" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K66" s="2" t="n">
-        <v>70</v>
-      </c>
-      <c r="L66" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>Chloé</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H67" t="n">
-        <v>20</v>
-      </c>
-      <c r="I67" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J67" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K67" s="2" t="n">
-        <v>71</v>
-      </c>
-      <c r="L67" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>Mr Bruno</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C68" t="n">
-        <v>1</v>
-      </c>
-      <c r="E68" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H68" t="n">
-        <v>20</v>
-      </c>
-      <c r="I68" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J68" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K68" s="2" t="n">
-        <v>72</v>
-      </c>
-      <c r="L68" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>Madame Bruno</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C69" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H69" t="n">
-        <v>20</v>
-      </c>
-      <c r="I69" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J69" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K69" s="2" t="n">
-        <v>73</v>
-      </c>
-      <c r="L69" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>Madcène</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C70" t="n">
-        <v>1</v>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H70" t="n">
-        <v>20</v>
-      </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J70" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K70" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="L70" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>Madina</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C71" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H71" t="n">
-        <v>20</v>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J71" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K71" s="2" t="n">
-        <v>75</v>
-      </c>
-      <c r="L71" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>Ermie</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C72" t="n">
-        <v>1</v>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E72" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F72" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H72" t="n">
-        <v>10</v>
-      </c>
-      <c r="I72" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J72" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K72" s="2" t="n">
-        <v>76</v>
-      </c>
-      <c r="L72" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>Numa Marie</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C73" t="n">
-        <v>1</v>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F73" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H73" t="n">
-        <v>20</v>
-      </c>
-      <c r="I73" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J73" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K73" s="2" t="n">
-        <v>77</v>
-      </c>
-      <c r="L73" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>Johnson</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C74" t="n">
-        <v>1</v>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>Poulet fricassé</t>
-        </is>
-      </c>
-      <c r="E74" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F74" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H74" t="n">
-        <v>20</v>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J74" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K74" s="2" t="n">
-        <v>78</v>
-      </c>
-      <c r="L74" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>Medson</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C75" t="n">
-        <v>1</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E75" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F75" t="inlineStr">
-        <is>
-          <t>Haricot vert</t>
-        </is>
-      </c>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H75" t="n">
-        <v>10</v>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J75" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K75" s="2" t="n">
-        <v>79</v>
-      </c>
-      <c r="L75" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>Sheskah</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C76" t="n">
-        <v>1</v>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E76" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F76" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H76" t="n">
-        <v>20</v>
-      </c>
-      <c r="I76" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J76" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K76" s="2" t="n">
-        <v>80</v>
-      </c>
-      <c r="L76" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Hélène Jean</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C77" t="n">
-        <v>1</v>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E77" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Haricot vert</t>
-        </is>
-      </c>
-      <c r="G77" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H77" t="n">
-        <v>10</v>
-      </c>
-      <c r="I77" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J77" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K77" s="2" t="n">
-        <v>81</v>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>Maman Lésimène</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C78" t="n">
-        <v>1</v>
-      </c>
-      <c r="D78" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H78" t="n">
-        <v>20</v>
-      </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J78" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K78" s="2" t="n">
-        <v>82</v>
-      </c>
-      <c r="L78" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>Rita Pierre</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C79" t="n">
-        <v>1</v>
-      </c>
-      <c r="D79" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="F79" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G79" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H79" t="n">
-        <v>20</v>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J79" s="1" t="n">
-        <v>20</v>
-      </c>
-      <c r="K79" s="2" t="n">
-        <v>84</v>
-      </c>
-      <c r="L79" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>Maturin</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>Famille</t>
-        </is>
-      </c>
-      <c r="C80" t="n">
-        <v>2</v>
-      </c>
-      <c r="D80" t="inlineStr">
-        <is>
-          <t>Crevette sauce poivrée</t>
-        </is>
-      </c>
-      <c r="E80" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="G80" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H80" t="n">
-        <v>20</v>
-      </c>
-      <c r="I80" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J80" s="1" t="n">
-        <v>40</v>
-      </c>
-      <c r="K80" s="2" t="n">
-        <v>85</v>
-      </c>
-      <c r="L80" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>Jean-Baptiste</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C81" t="n">
-        <v>1</v>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H81" t="n">
-        <v>10</v>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J81" s="1" t="n">
-        <v>10</v>
-      </c>
-      <c r="K81" s="2" t="n">
-        <v>86</v>
-      </c>
-      <c r="L81" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>Ursul Gurant</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C82" t="n">
-        <v>1</v>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Bœuf</t>
-        </is>
-      </c>
-      <c r="E82" t="inlineStr">
-        <is>
-          <t>Riz collé</t>
-        </is>
-      </c>
-      <c r="F82" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H82" t="n">
-        <v>20</v>
-      </c>
-      <c r="I82" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J82" t="n">
-        <v>10</v>
-      </c>
-      <c r="K82" t="n">
-        <v>87</v>
-      </c>
-      <c r="L82" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>Kimie</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>Individuel</t>
-        </is>
-      </c>
-      <c r="C83" t="n">
-        <v>1</v>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Travers de porc</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Riz blanc</t>
-        </is>
-      </c>
-      <c r="F83" t="inlineStr">
-        <is>
-          <t>Calalou</t>
-        </is>
-      </c>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Sur place</t>
-        </is>
-      </c>
-      <c r="H83" t="n">
-        <v>10</v>
-      </c>
-      <c r="I83" t="inlineStr">
-        <is>
-          <t>Non Payé</t>
-        </is>
-      </c>
-      <c r="J83" t="n">
-        <v>10</v>
-      </c>
-      <c r="K83" t="n">
-        <v>88</v>
-      </c>
-      <c r="L83" t="inlineStr">
-        <is>
-          <t>Non</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B87">
+  <conditionalFormatting sqref="B2:B89">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$L2="Oui"</formula>
     </cfRule>

</xml_diff>